<commit_message>
ajusta aba campos e melhora dropdown
</commit_message>
<xml_diff>
--- a/downloads/hr/output_automacao_hr.xlsx
+++ b/downloads/hr/output_automacao_hr.xlsx
@@ -7749,7 +7749,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:E22"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7767,9 +7767,6 @@
       <c r="E1" t="str">
         <v>campos</v>
       </c>
-      <c r="F1" t="str">
-        <v>tipo_campo</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -7787,76 +7784,64 @@
       <c r="E2" t="str">
         <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR; Elegiveis cota aprendiz (Count); F4; Fração p/ Empregado; Função Para Cota Sim; Matrícula</v>
       </c>
-      <c r="F2" t="str">
-        <v>Campo Calculado</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Horas Extras e Absenteísmo</v>
+        <v>Indicadores RH</v>
       </c>
       <c r="B3" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/HorasExtraseAbsentesmo/AnalticoHorasExtras</v>
+        <v>https://analyticsbi.sodexo.com.br/#/views/IndicadoresRH_16860832510040/IndicadoresdeRH</v>
       </c>
       <c r="C3" t="str">
-        <v>RH - Colaborador Folha; Elegiveis cota aprendiz (Tableau)</v>
+        <v>RH - Colaborador Folha; Elegiveis cota aprendiz (Tableau); EXPURGO_PEDIDO_DEMISSAO_FY24 Extração; METAS_HE_ABSENTEISMO; Other_KPIs_HR; Promoções_Internas</v>
       </c>
       <c r="D3" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/1057/lineage</v>
+        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/638/lineage</v>
       </c>
       <c r="E3" t="str">
-        <v/>
-      </c>
-      <c r="F3" t="str">
-        <v>Nao e Campo Calculado</v>
+        <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR; Elegiveis cota aprendiz (Count); F4; Fração p/ Empregado; Função Para Cota Sim; Matrícula; Expurgo Pedido Demissao; Extract (Count); Matricula; Diretoria; FY; METAS (Count); Segmento; Target Absenteismo; Target Horas Extras; :Measure Names; Absenteismo_Days (Count); Absenteismo_Days_Segmentos (Count); BRAZIL; CORPORATE; Data Compentecia; Data Competencia Womem; Days; Days (Absenteismo!Days!Segmentos); Dt Compentencia; Dt Competencia; Dt Competencia (Absenteismo!Days!Segmentos); Dt Competencia (Women Leardership); E&amp;R; EDUCATION; Filtro Absenteismo Segmentos; HEALTHCARE; KPI; Operacional; Other_KPIs_HR (Count); TARGET; Total; TRANSVERSAL; Women Leardership (Count); Promocoes; Promoções_Internas (Count)</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Indicadores RH</v>
+        <v>Base Colaboradores Geral</v>
       </c>
       <c r="B4" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/IndicadoresRH_16860832510040/IndicadoresdeRH</v>
+        <v>https://analyticsbi.sodexo.com.br/#/views/Basecolaboradoresgeral/Basecolaboradores</v>
       </c>
       <c r="C4" t="str">
-        <v>RH - Colaborador Folha; Elegiveis cota aprendiz (Tableau); EXPURGO_PEDIDO_DEMISSAO_FY24 Extração; METAS_HE_ABSENTEISMO; Other_KPIs_HR; Promoções_Internas</v>
+        <v>RH - Colaborador Folha</v>
       </c>
       <c r="D4" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/638/lineage</v>
+        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage</v>
       </c>
       <c r="E4" t="str">
-        <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR; Elegiveis cota aprendiz (Count); F4; Fração p/ Empregado; Função Para Cota Sim; Matrícula; Expurgo Pedido Demissao; Extract (Count); Matricula; Diretoria; FY; METAS (Count); Segmento; Target Absenteismo; Target Horas Extras; :Measure Names; Absenteismo_Days (Count); Absenteismo_Days_Segmentos (Count); BRAZIL; CORPORATE; Data Compentecia; Data Competencia Womem; Days; Days (Absenteismo!Days!Segmentos); Dt Compentencia; Dt Competencia; Dt Competencia (Absenteismo!Days!Segmentos); Dt Competencia (Women Leardership); E&amp;R; EDUCATION; Filtro Absenteismo Segmentos; HEALTHCARE; KPI; Operacional; Other_KPIs_HR (Count); TARGET; Total; TRANSVERSAL; Women Leardership (Count); Promocoes; Promoções_Internas (Count)</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Campo Calculado</v>
+        <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Indicadores RH</v>
+        <v>Indicadores DE&amp;I</v>
       </c>
       <c r="B5" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/IndicadoresRH_16860832510040/IndicadoresdeRH</v>
+        <v>https://analyticsbi.sodexo.com.br/#/views/IndicadoresDEI/TurnoverAbsentesmoHorasExtrasPcD</v>
       </c>
       <c r="C5" t="str">
-        <v>RH - Colaborador Folha; Elegiveis cota aprendiz (Tableau); EXPURGO_PEDIDO_DEMISSAO_FY24 Extração; METAS_HE_ABSENTEISMO; Other_KPIs_HR; Promoções_Internas</v>
+        <v>RH - Colaborador Folha | Projeto : Fonte de Dados Corporativa; RH - Promoção; tbElegibilidade_Cargo (db_Elegilidade_Cargos)</v>
       </c>
       <c r="D5" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/638/lineage</v>
+        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48036/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/1065/lineage</v>
       </c>
       <c r="E5" t="str">
-        <v/>
-      </c>
-      <c r="F5" t="str">
-        <v>Nao e Campo Calculado</v>
+        <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR; Cd Motivo Alteracao Grade; CEP; Cidade; Classificação HR Reporting; Cor Pele; Cpf; Ctps; Ctps Serie; DATABASE; Deficiencia; Dlg Dlsdesligamento; Cargo de Confiança; Categoria; Cota Aprendiz; Elegibilidade; Elegibilidade CBO; Grade; ID Elegibilidade Cota JA; Id Nível Hierárquico; Job Family; Job Family Group; Job Title - Inglês; Job Title - Português; Nível Hierárquico; Nível Superior; tbElegibilidade_Cargo (Count)</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Base Colaboradores Geral</v>
+        <v>Book de Indicadores de Pessoas</v>
       </c>
       <c r="B6" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/Basecolaboradoresgeral/Basecolaboradores</v>
+        <v>https://analyticsbi.sodexo.com.br/#/views/BookdeIndicadoresdePessoas/DashboardsdeRH</v>
       </c>
       <c r="C6" t="str">
         <v>RH - Colaborador Folha</v>
@@ -7867,76 +7852,64 @@
       <c r="E6" t="str">
         <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR</v>
       </c>
-      <c r="F6" t="str">
-        <v>Campo Calculado</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Base Colaboradores Geral</v>
+        <v>Projeto Ponto - Dashboard de Quantidade de Horas</v>
       </c>
       <c r="B7" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/Basecolaboradoresgeral/Basecolaboradores</v>
+        <v>https://analyticsbi.sodexo.com.br/#/views/ProjetoPonto-DashboarddeQuantidadedeHoras/ProjetoPonto-EventosAnaltico</v>
       </c>
       <c r="C7" t="str">
-        <v>RH - Colaborador Folha</v>
+        <v>RH - Colaborador Ponto Analitico RLS V2; RH - Colaborador Ponto Sintetico RLS; Ondas_Projeto_Ponto</v>
       </c>
       <c r="D7" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage</v>
+        <v>https://analyticsbi.sodexo.com.br/#/datasources/57887/lineage; https://analyticsbi.sodexo.com.br/#/datasources/58934/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/1275/lineage</v>
       </c>
       <c r="E7" t="str">
-        <v/>
-      </c>
-      <c r="F7" t="str">
-        <v>Nao e Campo Calculado</v>
+        <v>Cálculo1; Cálculo2; CD_BUSINESS_UNIT; COLAB_CBO; COLAB_CD_CARGO; COLAB_CD_ESTR_HIERAR; COLAB_CD_ESTR_HIERAR_COLAB; COLAB_CD_FILIAL_COLABORADOR; COLAB_CD_SINDICATO; COLAB_CD_SITUACAO; COLAB_COR_PELE; COLAB_CPF; COLAB_CTPS; COLAB_CTPS_SERIE; COLAB_DEFICIENCIA; COLAB_DLG_DLSDESLIGAMENTO; COLAB_DSC_CARGO; COLAB_DT_ADMISSAO; COLAB_DT_COMPETENCIA; COLAB_DT_FIM_CCUSTO; COLAB_DT_INICIO_AVISO_PREVIO; COLAB_DT_INICIO_CARGO; COLAB_DT_INICIO_CCUSTO; COLAB_DT_INICIO_SITUACAO; COLAB_DT_NASCIMENTO; COLAB_DT_PGTO_RESCISAO; COLAB_DT_REINTEGRACAO; COLAB_DT_RESCISAO; COLAB_E_MAIL; COLAB_ESTADO_CIVIL; COLAB_FLEG_CARGO_ELEGIVEL_JAPRENDIZ; COLAB_FLEG_ENQUADRAMENTO; COLAB_GESTOR; COLAB_GRADE; COLAB_GRAU_INSTRUCAO; COLAB_ID_FOLHA; COLAB_LOCAL; COLAB_MATRICULA; COLAB_MATRICULA_GESTOR; COLAB_MOTIVO_DESLIGAMENTO; COLAB_MOTIVO_REINTEGRACAO; COLAB_MUNICIPIO; CL; Clbr; Onda; Planilha1 (Count)</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Indicadores DE&amp;I</v>
+        <v>Base de Férias em Aberto</v>
       </c>
       <c r="B8" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/IndicadoresDEI/TurnoverAbsentesmoHorasExtrasPcD</v>
+        <v>https://analyticsbi.sodexo.com.br/#/views/Basedefriasemaberto/Basedefriasemaberto</v>
       </c>
       <c r="C8" t="str">
-        <v>RH - Colaborador Folha | Projeto : Fonte de Dados Corporativa; RH - Promoção; tbElegibilidade_Cargo (db_Elegilidade_Cargos)</v>
+        <v>RH - Colaborador Ponto Sintetico; RH - Programação de Férias</v>
       </c>
       <c r="D8" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48036/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/1065/lineage</v>
+        <v>https://analyticsbi.sodexo.com.br/#/datasources/17222/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48035/lineage</v>
       </c>
       <c r="E8" t="str">
-        <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR; Cd Motivo Alteracao Grade; CEP; Cidade; Classificação HR Reporting; Cor Pele; Cpf; Ctps; Ctps Serie; DATABASE; Deficiencia; Dlg Dlsdesligamento; Cargo de Confiança; Categoria; Cota Aprendiz; Elegibilidade; Elegibilidade CBO; Grade; ID Elegibilidade Cota JA; Id Nível Hierárquico; Job Family; Job Family Group; Job Title - Inglês; Job Title - Português; Nível Hierárquico; Nível Superior; tbElegibilidade_Cargo (Count)</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Campo Calculado</v>
+        <v>CD_BUSINESS_UNIT; COLAB_CBO; COLAB_CD_CARGO; COLAB_CD_ESTR_HIERAR; COLAB_CD_ESTR_HIERAR_COLAB; COLAB_CD_FILIAL_COLABORADOR; COLAB_CD_SINDICATO; COLAB_CD_SITUACAO; COLAB_COR_PELE; COLAB_CPF; COLAB_CTPS; COLAB_CTPS_SERIE; COLAB_DEFICIENCIA; COLAB_DLG_DLSDESLIGAMENTO; COLAB_DSC_CARGO; COLAB_DT_ADMISSAO; COLAB_DT_COMPETENCIA; COLAB_DT_FIM_CCUSTO; COLAB_DT_INICIO_AVISO_PREVIO; COLAB_DT_INICIO_CARGO; COLAB_DT_INICIO_CCUSTO; COLAB_DT_INICIO_SITUACAO; COLAB_DT_NASCIMENTO; COLAB_DT_PGTO_RESCISAO; COLAB_DT_REINTEGRACAO; COLAB_DT_RESCISAO; COLAB_E_MAIL; COLAB_ESTADO_CIVIL; COLAB_FLEG_CARGO_ELEGIVEL_JAPRENDIZ; COLAB_FLEG_ENQUADRAMENTO; COLAB_GESTOR; COLAB_GRADE; COLAB_GRAU_INSTRUCAO; COLAB_ID_FOLHA; COLAB_LOCAL; COLAB_MATRICULA; COLAB_MATRICULA_GESTOR; COLAB_MOTIVO_DESLIGAMENTO; COLAB_MOTIVO_REINTEGRACAO; COLAB_MUNICIPIO; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cardapio; Cd Cargo; Cd Cargo HR Reporting; Cd Centro Custo; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Empresa Sodexo; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Filial Ficticia; Cd Grupoeconomico; Cd Matricula Diretor Operac; Cd Matricula Gerente Area; Cd Matricula Gerente Regional; Cd Matriz; Cd Período Descanso; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd Status; Cd Tipo Atuacao; Cd Tipo Contrato; Cd Tipo Servico; Cd Uf; CD_HORARIO; CD_TP_FILIAL_COLABORADOR; Classificação HR Reporting; Cor Pele; Cpf; Ctps; Ctps Serie; DATABASE</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Indicadores DE&amp;I</v>
+        <v>Modelo de Trabalho</v>
       </c>
       <c r="B9" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/IndicadoresDEI/TurnoverAbsentesmoHorasExtrasPcD</v>
+        <v>https://analyticsbi.sodexo.com.br/#/views/ModelodeTrabalho/ModelodeTrabalho</v>
       </c>
       <c r="C9" t="str">
-        <v>RH - Colaborador Folha | Projeto : Fonte de Dados Corporativa; RH - Promoção; tbElegibilidade_Cargo (db_Elegilidade_Cargos)</v>
+        <v>RH - Colaborador Folha</v>
       </c>
       <c r="D9" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48036/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/1065/lineage</v>
+        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage</v>
       </c>
       <c r="E9" t="str">
-        <v/>
-      </c>
-      <c r="F9" t="str">
-        <v>Nao e Campo Calculado</v>
+        <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Book de Indicadores de Pessoas</v>
+        <v>Banco de Horas</v>
       </c>
       <c r="B10" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/BookdeIndicadoresdePessoas/DashboardsdeRH</v>
+        <v>https://analyticsbi.sodexo.com.br/#/views/Bancodehoras/Bancodehoras</v>
       </c>
       <c r="C10" t="str">
         <v>RH - Colaborador Folha</v>
@@ -7947,176 +7920,149 @@
       <c r="E10" t="str">
         <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR</v>
       </c>
-      <c r="F10" t="str">
-        <v>Campo Calculado</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Book de Indicadores de Pessoas</v>
+        <v>Metas Turnover FY25 - Regrettable e Demissional</v>
       </c>
       <c r="B11" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/BookdeIndicadoresdePessoas/DashboardsdeRH</v>
+        <v>https://analyticsbi.sodexo.com.br/#/views/MetasTurnoverFY25-RegrettableBoostereDemissional/METASDERHFY25</v>
       </c>
       <c r="C11" t="str">
-        <v>RH - Colaborador Folha</v>
+        <v>RH - Colaborador Folha; Elegiveis cota aprendiz (Tableau); EXPURGO_PEDIDO_DEMISSAO_FY24 Extração; METAS_HE_ABSENTEISMO; Other_KPIs_HR; Promoções_Internas</v>
       </c>
       <c r="D11" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage</v>
+        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/1853/lineage</v>
       </c>
       <c r="E11" t="str">
-        <v/>
-      </c>
-      <c r="F11" t="str">
-        <v>Nao e Campo Calculado</v>
+        <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR; Elegiveis cota aprendiz (Count); F4; Fração p/ Empregado; Função Para Cota Sim; Matrícula; Expurgo Pedido Demissao; Extract (Count); Matricula; Diretoria; FY; METAS (Count); Segmento; Target Absenteismo; Target Horas Extras; :Measure Names; Absenteismo_Days (Count); Absenteismo_Days_Segmentos (Count); BRAZIL; CORPORATE; Data Compentecia; Data Competencia Womem; Days; Days (Absenteismo!Days!Segmentos); Dt Compentencia; Dt Competencia; Dt Competencia (Absenteismo!Days!Segmentos); Dt Competencia (Women Leardership); E&amp;R; EDUCATION; Filtro Absenteismo Segmentos; HEALTHCARE; KPI; Operacional; Other_KPIs_HR (Count); TARGET; Total; TRANSVERSAL; Women Leardership (Count); Promocoes; Promoções_Internas (Count)</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Projeto Ponto - Dashboard de Quantidade de Horas</v>
+        <v>Metas Turnover FY26 - Regrettable e Demissional</v>
       </c>
       <c r="B12" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/ProjetoPonto-DashboarddeQuantidadedeHoras/ProjetoPonto-EventosAnaltico</v>
+        <v>https://analyticsbi.sodexo.com.br/#/views/MetasTurnoverFY26-RegrettableeDemissional/MetasdeRHFY26</v>
       </c>
       <c r="C12" t="str">
-        <v>RH - Colaborador Ponto Analitico RLS V2; RH - Colaborador Ponto Sintetico RLS; Ondas_Projeto_Ponto</v>
+        <v/>
       </c>
       <c r="D12" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/57887/lineage; https://analyticsbi.sodexo.com.br/#/datasources/58934/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/1275/lineage</v>
+        <v>ERRO: O painel nao pode ser acessado com a sessao atual no Tableau.</v>
       </c>
       <c r="E12" t="str">
-        <v>Cálculo1; Cálculo2; CD_BUSINESS_UNIT; COLAB_CBO; COLAB_CD_CARGO; COLAB_CD_ESTR_HIERAR; COLAB_CD_ESTR_HIERAR_COLAB; COLAB_CD_FILIAL_COLABORADOR; COLAB_CD_SINDICATO; COLAB_CD_SITUACAO; COLAB_COR_PELE; COLAB_CPF; COLAB_CTPS; COLAB_CTPS_SERIE; COLAB_DEFICIENCIA; COLAB_DLG_DLSDESLIGAMENTO; COLAB_DSC_CARGO; COLAB_DT_ADMISSAO; COLAB_DT_COMPETENCIA; COLAB_DT_FIM_CCUSTO; COLAB_DT_INICIO_AVISO_PREVIO; COLAB_DT_INICIO_CARGO; COLAB_DT_INICIO_CCUSTO; COLAB_DT_INICIO_SITUACAO; COLAB_DT_NASCIMENTO; COLAB_DT_PGTO_RESCISAO; COLAB_DT_REINTEGRACAO; COLAB_DT_RESCISAO; COLAB_E_MAIL; COLAB_ESTADO_CIVIL; COLAB_FLEG_CARGO_ELEGIVEL_JAPRENDIZ; COLAB_FLEG_ENQUADRAMENTO; COLAB_GESTOR; COLAB_GRADE; COLAB_GRAU_INSTRUCAO; COLAB_ID_FOLHA; COLAB_LOCAL; COLAB_MATRICULA; COLAB_MATRICULA_GESTOR; COLAB_MOTIVO_DESLIGAMENTO; COLAB_MOTIVO_REINTEGRACAO; COLAB_MUNICIPIO; CL; Clbr; Onda; Planilha1 (Count)</v>
-      </c>
-      <c r="F12" t="str">
-        <v>Campo Calculado</v>
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Projeto Ponto - Dashboard de Quantidade de Horas</v>
+        <v>Women Leadership</v>
       </c>
       <c r="B13" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/ProjetoPonto-DashboarddeQuantidadedeHoras/ProjetoPonto-EventosAnaltico</v>
+        <v>https://analyticsbi.sodexo.com.br/#/views/WomenLeadership/IndicadoresWomenLeadership</v>
       </c>
       <c r="C13" t="str">
-        <v>RH - Colaborador Ponto Analitico RLS V2; RH - Colaborador Ponto Sintetico RLS; Ondas_Projeto_Ponto</v>
+        <v/>
       </c>
       <c r="D13" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/57887/lineage; https://analyticsbi.sodexo.com.br/#/datasources/58934/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/1275/lineage</v>
+        <v>ERRO: Nao encontrei o link do workbook no painel Data Details.</v>
       </c>
       <c r="E13" t="str">
         <v/>
-      </c>
-      <c r="F13" t="str">
-        <v>Nao e Campo Calculado</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Base de Férias em Aberto</v>
+        <v>Wokforce Planning</v>
       </c>
       <c r="B14" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/Basedefriasemaberto/Basedefriasemaberto</v>
+        <v>https://analyticsbi.sodexo.com.br/#/views/WokforcePlanning/WorkforcePlanning</v>
       </c>
       <c r="C14" t="str">
-        <v>RH - Colaborador Ponto Sintetico; RH - Programação de Férias</v>
+        <v>RH - Colaborador Folha; DE-PARA_BU; Elegiveis cota aprendiz (Tableau); EXPURGO_PEDIDO_DEMISSAO_FY24 Extração; METAS_HE_ABSENTEISMO; Other_KPIs_HR; Promoções_Internas</v>
       </c>
       <c r="D14" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/17222/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48035/lineage</v>
+        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/2103/lineage</v>
       </c>
       <c r="E14" t="str">
-        <v/>
-      </c>
-      <c r="F14" t="str">
-        <v>Campo Calculado</v>
+        <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR; CL; DE PARA (Count); Diretoria; Nome do Centro de Lucro; Nome do Grupo Economico; Nome TLR; Nome TLR-1; Nome TLR-2; Nome TLR-3; Para BU; Para BU SAP; Para Diretoria; Para Diretoria SAP; Para Portfólio; Para Portfólio SAP; Para TLR; Para TLR-1; Para TLR-2; Para TLR-3; Para TLR BU; Portfólio; Segmento; Elegiveis cota aprendiz (Count); F4; Fração p/ Empregado; Função Para Cota Sim; Matrícula; Expurgo Pedido Demissao; Extract (Count); Matricula; FY; METAS (Count); Target Absenteismo; Target Horas Extras; :Measure Names; Absenteismo_Days (Count); Absenteismo_Days_Segmentos (Count); BRAZIL; CORPORATE; Data Compentecia; Data Competencia Womem; Days; Days (Absenteismo!Days!Segmentos); Dt Compentencia; Dt Competencia; Dt Competencia (Absenteismo!Days!Segmentos); Dt Competencia (Women Leardership); E&amp;R; EDUCATION; Filtro Absenteismo Segmentos; HEALTHCARE; KPI; Operacional; Other_KPIs_HR (Count); TARGET; Total; TRANSVERSAL; Women Leardership (Count); Promocoes; Promoções_Internas (Count)</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Base de Férias em Aberto</v>
+        <v>Indicadores de Chamados e Workflows</v>
       </c>
       <c r="B15" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/Basedefriasemaberto/Basedefriasemaberto</v>
+        <v>https://analyticsbi.sodexo.com.br/#/views/IndicadoresdeChamadoseWorkflows/Painel0-Home</v>
       </c>
       <c r="C15" t="str">
-        <v>RH - Colaborador Ponto Sintetico; RH - Programação de Férias</v>
+        <v>dCalendario; fChamadosEmAberto; fChamadosResolvidos; fWorkflowsEmAberto; fWorkflowsResolvidos</v>
       </c>
       <c r="D15" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/17222/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48035/lineage</v>
+        <v>https://analyticsbi.sodexo.com.br/#/workbooks/2227/lineage</v>
       </c>
       <c r="E15" t="str">
-        <v>CD_BUSINESS_UNIT; COLAB_CBO; COLAB_CD_CARGO; COLAB_CD_ESTR_HIERAR; COLAB_CD_ESTR_HIERAR_COLAB; COLAB_CD_FILIAL_COLABORADOR; COLAB_CD_SINDICATO; COLAB_CD_SITUACAO; COLAB_COR_PELE; COLAB_CPF; COLAB_CTPS; COLAB_CTPS_SERIE; COLAB_DEFICIENCIA; COLAB_DLG_DLSDESLIGAMENTO; COLAB_DSC_CARGO; COLAB_DT_ADMISSAO; COLAB_DT_COMPETENCIA; COLAB_DT_FIM_CCUSTO; COLAB_DT_INICIO_AVISO_PREVIO; COLAB_DT_INICIO_CARGO; COLAB_DT_INICIO_CCUSTO; COLAB_DT_INICIO_SITUACAO; COLAB_DT_NASCIMENTO; COLAB_DT_PGTO_RESCISAO; COLAB_DT_REINTEGRACAO; COLAB_DT_RESCISAO; COLAB_E_MAIL; COLAB_ESTADO_CIVIL; COLAB_FLEG_CARGO_ELEGIVEL_JAPRENDIZ; COLAB_FLEG_ENQUADRAMENTO; COLAB_GESTOR; COLAB_GRADE; COLAB_GRAU_INSTRUCAO; COLAB_ID_FOLHA; COLAB_LOCAL; COLAB_MATRICULA; COLAB_MATRICULA_GESTOR; COLAB_MOTIVO_DESLIGAMENTO; COLAB_MOTIVO_REINTEGRACAO; COLAB_MUNICIPIO; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cardapio; Cd Cargo; Cd Cargo HR Reporting; Cd Centro Custo; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Empresa Sodexo; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Filial Ficticia; Cd Grupoeconomico; Cd Matricula Diretor Operac; Cd Matricula Gerente Area; Cd Matricula Gerente Regional; Cd Matriz; Cd Período Descanso; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd Status; Cd Tipo Atuacao; Cd Tipo Contrato; Cd Tipo Servico; Cd Uf; CD_HORARIO; CD_TP_FILIAL_COLABORADOR; Classificação HR Reporting; Cor Pele; Cpf; Ctps; Ctps Serie; DATABASE</v>
-      </c>
-      <c r="F15" t="str">
-        <v>Nao e Campo Calculado</v>
+        <v>Ano; Ano Fiscal; Data; Dia; Dia da Semana; Dia da Semana ID; Extract (Count); Fiscal Year; Mês; Mês Abr; Mês Fiscal; Mês ID; Mês/Ano; Mês/Ano ID; Período Fiscal ID; Período/FY; Período/FY ID; Semana do Ano; Semana do Ano ID; Semana Fiscal do Ano; Semana Fiscal do Ano ID; Semana Fiscal/Ano ID; Semana/Ano; Semana/Ano ID; Semestre Fiscal / Ano ID; Semestre Fiscal do Ano; Semestre ID; Trimestre Fiscal; Trimestre Fiscal/Ano; Trimestre Fiscal/Ano ID; Assunto; Atribuído ao Usuário; Criador; Data de Conclusão Alvo; Data de Criação; Data Referência; Em nome de; Equipe Atribuída; Fila Atribuída; Fonte; Horas SLA; ID do caso; ID do Caso Relacionado; Prioridade; Solicitado por; Status do caso; Subtópico de RH; Tema de RH; % No Prazo; :Measure Names; Atingiu a Meta; Data de Conclusão Alvo Ajustada; Data de reabertura; Data Referência Resolução; Data/Hora da Primeira Resposta; Data/Hora Resolvida; Dia da Semana Criação; Fila Atribuída (Subequipe); Meta; Número do chamado; Período Fiscal; Qtde Em Atraso; Qtde No Prazo; Reabertos; Status do chamado; Status Prazo Primeiro Atendimento; Tempo de Resolução do Caso (Dias Úteis); Tempo de Trabalho em Dias Úteis; Tempo de trabalho em horas úteis (até agora); Total Atendimentos; Data da Etapa; Data prazo atendimento; Data Referencia; Data/hora início da transação; Dentro do prazo?; Equipe; Etapa de Workflow; Feriado; Formulário de Workflow; Id etapa de workflow; Id Formulário de Workflow; Id Lançamento de Workflow; Nome do Usuário; Referência; Solicitante; Subequipe; % Dentro do Prazo; Atendido Em; Categoria Dia Entrada Wf; Categoria Dia Prazo Atend; Data Prazo Atendimento 2; Data Rescisão; Dentro Prazo?; Efetivado?; Entrada Wf; Entrada Wf 2; Etapa Destino; Etapa Origem; Etapa Wf - Destino; Etapa Wf - Origem; Formulário Wf; Grupo Usuário; Id Formulário Wf; Id Grupo Usuário; Id Log Transação Wf; Id Workflow; Meta WFs; Nome Usuário; Novo Status Dentro Prazo; Prazo Atendimento 1º Dia Útil Próximo Mês; Prazo Atendimento Exceto Abertura Fim De Mês; Qtde Dentro do Prazo; Qtde Fora do Prazo; Status da Meta; Superior Hierárquico; Tempo Atendim Horas Uteis; Tempo Atendimento Hr</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Modelo de Trabalho</v>
+        <v>Visão consolidada</v>
       </c>
       <c r="B16" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/ModelodeTrabalho/ModelodeTrabalho</v>
+        <v>https://analyticsbi.sodexo.com.br/#/views/Visoconsolidada/Consolidadodedados</v>
       </c>
       <c r="C16" t="str">
-        <v>RH - Colaborador Folha</v>
+        <v>RH - Colaborador Folha; Elegiveis cota aprendiz (Tableau); PCD (Tableau)</v>
       </c>
       <c r="D16" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage</v>
+        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/700/lineage</v>
       </c>
       <c r="E16" t="str">
-        <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR</v>
-      </c>
-      <c r="F16" t="str">
-        <v>Campo Calculado</v>
+        <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR; Elegiveis cota aprendiz (Count); Fração p/ Empregado; Função Para Cota Sim; Matrícula; PCD (Count); Qtd. Pcd</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Modelo de Trabalho</v>
+        <v>Zona Posicionamento Salarial</v>
       </c>
       <c r="B17" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/ModelodeTrabalho/ModelodeTrabalho</v>
+        <v>https://analyticsbi.sodexo.com.br/#/views/ZonaPosicionamentoSalarial/ZonasdePosicionamentoSalarial</v>
       </c>
       <c r="C17" t="str">
-        <v>RH - Colaborador Folha</v>
+        <v>RH - Base_Enios_Tableau; RH - Colaborador Folha</v>
       </c>
       <c r="D17" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage</v>
+        <v>https://analyticsbi.sodexo.com.br/#/datasources/52187/lineage; https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage</v>
       </c>
       <c r="E17" t="str">
-        <v/>
-      </c>
-      <c r="F17" t="str">
-        <v>Nao e Campo Calculado</v>
+        <v>Admissão; Cargo; CL; Colaborador; Cpf; Dados gerados em; Diretoria; Dt Competencia; Dt inic cargo atual; Dt nasc; Gênero; Gestor; Grade; HR Reporting; Matrícula; Munic. cl; Nome do cl; Portfolio; Posição Faixa; Região cl; Segmento; Situação; Tipo cl; Uf cl; Zona posicionamento; % Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Banco de Horas</v>
+        <v>Base de Dados Modelo de Trabalho - Home Office</v>
       </c>
       <c r="B18" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/Bancodehoras/Bancodehoras</v>
+        <v>https://analyticsbi.sodexo.com.br/#/views/BasedeDadosModelodeTrabalho-HomeOffice/BASEOFICIALPARATABLEAU</v>
       </c>
       <c r="C18" t="str">
-        <v>RH - Colaborador Folha</v>
+        <v>RH - Colaborador Folha; RH - Programação de Férias; RH STEP Afastamento; Base_Catracas; Base_Tableau; reserva_mesas_por_colaborador geral</v>
       </c>
       <c r="D18" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage</v>
+        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48035/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48064/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/2183/lineage</v>
       </c>
       <c r="E18" t="str">
-        <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR</v>
-      </c>
-      <c r="F18" t="str">
-        <v>Campo Calculado</v>
+        <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR; Cd Cardapio; Cd Centro Custo; Cd Empresa Sodexo; Cd Filial Ficticia; Cd Grupoeconomico; Cd Matricula Diretor Operac; Cd Matricula Gerente Area; Cd Matricula Gerente Regional; Cd Matriz; Cd Período Descanso; Cd Status; Cd Tipo Atuacao; Cd Tipo Servico; Cd Uf; Classificação HR Reporting; Cor Pele; Cpf; Ctps; Ctps Serie; DATABASE; AFAST_CARGO; AFAST_CD_FILIAL; AFAST_CD_SITUACAO; AFAST_CID_DOENCA; AFAST_CID_DOENCA_OFICIAL; AFAST_DSC_DOENCA; AFAST_DSC_MOTIVO_SITUACAO; AFAST_DT_CARGA; AFAST_DT_COMPETENCIA; AFAST_DT_FIM; AFAST_DT_INICIO; AFAST_MATRICULA; AFAST_MOTIVO; AFAST_QT_DIAS_AFASTAMENTO; AFAST_QT_DIAS_AFASTAMENTO_STEP; AFAST_SITUACAO; Competencia; Data Acesso; Email; Empresa; Eqp Id; Equipamento; ES; Hora Acesso; Matricula; Nome; Planilha1 (Count); Qt Acessos; % Conformidade Hibrido Dentro da Meta; % Conformidade Hibrido Fora da Meta; % Conformidade Home 100%; % Conformidade Home Geral; % Conformidade Home Hibrido; :Measure Names; Analise Qt Check-in; Analise Qt Check-in 2; Base_Tableau (Count); Business Unit; Competência; Cor Conformidade; Dias de afastamento no mês; Dias de férias no mês; Dsc Cargo; Dt Admissao; Elegiveis por UF; Email Gestor; Flag Last 6 Month; Flag Mes Atual; Gestor; Matricula Gestor; Modelo de Trabalho; Nm Diretoria; Nm Filial; Nm Segmento; Nome Colaborador; Qt Check-in; Qt Check-in Filtro; Qt Colab Divergente Home 100%; Qt Colab Divergente Home Hibrido; Qt Colaboradores; Qt Colaboradores Filtro; Qt de Check-in; Qt Home Office 100%; Qt Home Office 100% em conformidade; Qt Home Office 100% Não conformidade; Qt Home Office em conformidade; Andar; Cancelado por; Check-in &lt;4; Check-in realizado; Check-out realizado; Data da solicitação; Data de cancelamento; Data do check-in; Data do check-out; Data final; Data inicial; E-mail; Id; Mesa; Plan1 (Count); Planta; Qt Checkin Home Office 100% Divergente; Qt Colab Home Office 100% Divergente; Qt Colab Home Office Hibrido Divergente; Qt de Checkin; Qt Errada Hibrido; Status; Tirou férias no mês?; Total de Check-in; Total de Check-in DIM; Total de Checkin</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Banco de Horas</v>
+        <v>Indicadores de Promoções Internas</v>
       </c>
       <c r="B19" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/Bancodehoras/Bancodehoras</v>
+        <v>https://analyticsbi.sodexo.com.br/#/views/IndicadoresdePromoesInternas/PromoesInternas</v>
       </c>
       <c r="C19" t="str">
         <v>RH - Colaborador Folha</v>
@@ -8125,495 +8071,63 @@
         <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage</v>
       </c>
       <c r="E19" t="str">
-        <v/>
-      </c>
-      <c r="F19" t="str">
-        <v>Nao e Campo Calculado</v>
+        <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Metas Turnover FY25 - Regrettable e Demissional</v>
+        <v>Indicadores de Modelo de Trabalho - Home Office</v>
       </c>
       <c r="B20" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/MetasTurnoverFY25-RegrettableBoostereDemissional/METASDERHFY25</v>
+        <v>https://analyticsbi.sodexo.com.br/#/views/IndicadoresdeModelodeTrabalho-HomeOffice_17522412067850/DashboardHomeOffice-Colaboradores</v>
       </c>
       <c r="C20" t="str">
-        <v>RH - Colaborador Folha; Elegiveis cota aprendiz (Tableau); EXPURGO_PEDIDO_DEMISSAO_FY24 Extração; METAS_HE_ABSENTEISMO; Other_KPIs_HR; Promoções_Internas</v>
+        <v>RH - Colaborador Folha; RH - Programação de Férias; RH STEP Afastamento; Base_Tableau; reserva_mesas_por_colaborador geral</v>
       </c>
       <c r="D20" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/1853/lineage</v>
+        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48035/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48064/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/2169/lineage</v>
       </c>
       <c r="E20" t="str">
-        <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR; Elegiveis cota aprendiz (Count); F4; Fração p/ Empregado; Função Para Cota Sim; Matrícula; Expurgo Pedido Demissao; Extract (Count); Matricula; Diretoria; FY; METAS (Count); Segmento; Target Absenteismo; Target Horas Extras; :Measure Names; Absenteismo_Days (Count); Absenteismo_Days_Segmentos (Count); BRAZIL; CORPORATE; Data Compentecia; Data Competencia Womem; Days; Days (Absenteismo!Days!Segmentos); Dt Compentencia; Dt Competencia; Dt Competencia (Absenteismo!Days!Segmentos); Dt Competencia (Women Leardership); E&amp;R; EDUCATION; Filtro Absenteismo Segmentos; HEALTHCARE; KPI; Operacional; Other_KPIs_HR (Count); TARGET; Total; TRANSVERSAL; Women Leardership (Count); Promocoes; Promoções_Internas (Count)</v>
-      </c>
-      <c r="F20" t="str">
-        <v>Campo Calculado</v>
+        <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR; Cd Cardapio; Cd Centro Custo; Cd Empresa Sodexo; Cd Filial Ficticia; Cd Grupoeconomico; Cd Matricula Diretor Operac; Cd Matricula Gerente Area; Cd Matricula Gerente Regional; Cd Matriz; Cd Período Descanso; Cd Status; Cd Tipo Atuacao; Cd Tipo Servico; Cd Uf; Classificação HR Reporting; Cor Pele; Cpf; Ctps; Ctps Serie; DATABASE; AFAST_CARGO; AFAST_CD_FILIAL; AFAST_CD_SITUACAO; AFAST_CID_DOENCA; AFAST_CID_DOENCA_OFICIAL; AFAST_DSC_DOENCA; AFAST_DSC_MOTIVO_SITUACAO; AFAST_DT_CARGA; AFAST_DT_COMPETENCIA; AFAST_DT_FIM; AFAST_DT_INICIO; AFAST_MATRICULA; AFAST_MOTIVO; AFAST_QT_DIAS_AFASTAMENTO; AFAST_QT_DIAS_AFASTAMENTO_STEP; AFAST_SITUACAO; % Conformidade Hibrido Dentro da Meta; % Conformidade Hibrido Fora da Meta; % Conformidade Home 100%; % Conformidade Home Geral; % Conformidade Home Hibrido; :Measure Names; Analise Qt Check-in; Analise Qt Check-in 2; Base_Tableau (Count); Business Unit; Competência; Cor Conformidade; Dias de afastamento no mês; Dias de férias no mês; Dsc Cargo; Dt Admissao; Elegiveis por UF; Email Gestor; Flag Last 6 Month; Flag Mes Atual; Gestor; Matricula; Matricula Gestor; Modelo de Trabalho; Nm Diretoria; Nm Filial; Nm Segmento; Nome Colaborador; Qt Check-in; Qt Check-in Filtro; Qt Colab Divergente Home 100%; Qt Colab Divergente Home Hibrido; Qt Colaboradores; Qt Colaboradores Filtro; Qt de Check-in; Qt Home Office 100%; Qt Home Office 100% em conformidade; Qt Home Office 100% Não conformidade; Qt Home Office em conformidade; Andar; Cancelado por; Check-in &lt;4; Check-in realizado; Check-out realizado; Competencia; Data da solicitação; Data de cancelamento; Data do check-in; Data do check-out; Data final; Data inicial; E-mail; Id; Mesa; Nome; Plan1 (Count); Planta; Qt Checkin Home Office 100% Divergente; Qt Colab Home Office 100% Divergente; Qt Colab Home Office Hibrido Divergente; Qt Errada Hibrido; Status; Tirou férias no mês?; Total de Check-in; Total de Check-in DIM; Total de Checkin</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Metas Turnover FY25 - Regrettable e Demissional</v>
+        <v>Painel de Vagas Operacionais</v>
       </c>
       <c r="B21" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/MetasTurnoverFY25-RegrettableBoostereDemissional/METASDERHFY25</v>
+        <v>https://analyticsbi.sodexo.com.br/#/views/PaineldeVagasOperacionais/AnlisesdeVagasOperacionais</v>
       </c>
       <c r="C21" t="str">
-        <v>RH - Colaborador Folha; Elegiveis cota aprendiz (Tableau); EXPURGO_PEDIDO_DEMISSAO_FY24 Extração; METAS_HE_ABSENTEISMO; Other_KPIs_HR; Promoções_Internas</v>
+        <v>BIVARREDURA - Filial; RH - Colaborador Folha; RH STEP Abertura de Vagas</v>
       </c>
       <c r="D21" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/1853/lineage</v>
+        <v>https://analyticsbi.sodexo.com.br/#/datasources/23931/lineage; https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48063/lineage</v>
       </c>
       <c r="E21" t="str">
-        <v/>
-      </c>
-      <c r="F21" t="str">
-        <v>Nao e Campo Calculado</v>
+        <v>[END] Bairro; [END] CEP; [END] Cidade; [END] LATITUDE; [END] Logadouro; [END] LONGITUDE; [END] UF; Cd Cardapio; Cd Centro Custo; Cd Diretoria; Cd Empresa Sodexo; Cd Filial; Cd Filial Ficticia; Cd Grupo Economico; Cd Matricula Diretor Operac; Cd Matricula Gerente Area; Cd Matricula Gerente Regional; Cd Matriz; Cd Regional; Cd Segmento; Cd Tipo Atuacao; Cd Tipo Contrato; Cd Tipo Servico; Cd Uf; CD_BUSINESS_UNIT; Dados migrados (Count); Dt Abertura; Dt Encerramento; Fili Email; Fl Ficticia; Inscricaoestadual; Nm Bairro; Nm Cardapio; Nm Cidade; Nm Diretor Operacional; Nm Diretoria; Nm Empresa Sodexo; Nm Filial; Nm Gerente Area; Nm Gerente Regional; % Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial Colaborador; Cd Grupo CL; Cd Matriz Cardapio; Cd Matriz Compras; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR; Cd Portfolio; CD_CARGO; CD_CARGO_HR_REPORTING; CD_CARGO_VAGA; CD_COTA_APRENDIZ_CBO; CD_ESTR_HIERAR; CD_ESTR_HIERAR_COLAB; CD_FILIAL_COLABORADOR; CD_FILIAL_VAGA; CD_FLEXIVEL_VAGA; CD_SINDICATO; CD_SITUACAO; CD_VAGA; CLASSIFICACAO_HR_REPORTING; COR_PELE; CPF; CTPS</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Metas Turnover FY26 - Regrettable e Demissional</v>
+        <v>Pin People On e Off</v>
       </c>
       <c r="B22" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/MetasTurnoverFY26-RegrettableeDemissional/MetasdeRHFY26</v>
+        <v>https://analyticsbi.sodexo.com.br/#/views/PinPeopleOneOff/PinPeople</v>
       </c>
       <c r="C22" t="str">
-        <v/>
+        <v>RH - Colaborador Folha | Projeto : Fonte de Dados Corporativa; tbElegibilidade_Cargo (db_Elegilidade_Cargos)</v>
       </c>
       <c r="D22" t="str">
-        <v>ERRO: O painel nao pode ser acessado com a sessao atual no Tableau.</v>
+        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/1009/lineage</v>
       </c>
       <c r="E22" t="str">
-        <v/>
-      </c>
-      <c r="F22" t="str">
-        <v>Campo Calculado</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>Metas Turnover FY26 - Regrettable e Demissional</v>
-      </c>
-      <c r="B23" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/MetasTurnoverFY26-RegrettableeDemissional/MetasdeRHFY26</v>
-      </c>
-      <c r="C23" t="str">
-        <v/>
-      </c>
-      <c r="D23" t="str">
-        <v>ERRO: O painel nao pode ser acessado com a sessao atual no Tableau.</v>
-      </c>
-      <c r="E23" t="str">
-        <v/>
-      </c>
-      <c r="F23" t="str">
-        <v>Nao e Campo Calculado</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>Women Leadership</v>
-      </c>
-      <c r="B24" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/WomenLeadership/IndicadoresWomenLeadership</v>
-      </c>
-      <c r="C24" t="str">
-        <v/>
-      </c>
-      <c r="D24" t="str">
-        <v>ERRO: Nao encontrei o link do workbook no painel Data Details.</v>
-      </c>
-      <c r="E24" t="str">
-        <v/>
-      </c>
-      <c r="F24" t="str">
-        <v>Campo Calculado</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>Women Leadership</v>
-      </c>
-      <c r="B25" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/WomenLeadership/IndicadoresWomenLeadership</v>
-      </c>
-      <c r="C25" t="str">
-        <v/>
-      </c>
-      <c r="D25" t="str">
-        <v>ERRO: Nao encontrei o link do workbook no painel Data Details.</v>
-      </c>
-      <c r="E25" t="str">
-        <v/>
-      </c>
-      <c r="F25" t="str">
-        <v>Nao e Campo Calculado</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>Wokforce Planning</v>
-      </c>
-      <c r="B26" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/WokforcePlanning/WorkforcePlanning</v>
-      </c>
-      <c r="C26" t="str">
-        <v>RH - Colaborador Folha; DE-PARA_BU; Elegiveis cota aprendiz (Tableau); EXPURGO_PEDIDO_DEMISSAO_FY24 Extração; METAS_HE_ABSENTEISMO; Other_KPIs_HR; Promoções_Internas</v>
-      </c>
-      <c r="D26" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/2103/lineage</v>
-      </c>
-      <c r="E26" t="str">
-        <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR; CL; DE PARA (Count); Diretoria; Nome do Centro de Lucro; Nome do Grupo Economico; Nome TLR; Nome TLR-1; Nome TLR-2; Nome TLR-3; Para BU; Para BU SAP; Para Diretoria; Para Diretoria SAP; Para Portfólio; Para Portfólio SAP; Para TLR; Para TLR-1; Para TLR-2; Para TLR-3; Para TLR BU; Portfólio; Segmento; Elegiveis cota aprendiz (Count); F4; Fração p/ Empregado; Função Para Cota Sim; Matrícula; Expurgo Pedido Demissao; Extract (Count); Matricula; FY; METAS (Count); Target Absenteismo; Target Horas Extras; :Measure Names; Absenteismo_Days (Count); Absenteismo_Days_Segmentos (Count); BRAZIL; CORPORATE; Data Compentecia; Data Competencia Womem; Days; Days (Absenteismo!Days!Segmentos); Dt Compentencia; Dt Competencia; Dt Competencia (Absenteismo!Days!Segmentos); Dt Competencia (Women Leardership); E&amp;R; EDUCATION; Filtro Absenteismo Segmentos; HEALTHCARE; KPI; Operacional; Other_KPIs_HR (Count); TARGET; Total; TRANSVERSAL; Women Leardership (Count); Promocoes; Promoções_Internas (Count)</v>
-      </c>
-      <c r="F26" t="str">
-        <v>Campo Calculado</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>Wokforce Planning</v>
-      </c>
-      <c r="B27" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/WokforcePlanning/WorkforcePlanning</v>
-      </c>
-      <c r="C27" t="str">
-        <v>RH - Colaborador Folha; DE-PARA_BU; Elegiveis cota aprendiz (Tableau); EXPURGO_PEDIDO_DEMISSAO_FY24 Extração; METAS_HE_ABSENTEISMO; Other_KPIs_HR; Promoções_Internas</v>
-      </c>
-      <c r="D27" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/2103/lineage</v>
-      </c>
-      <c r="E27" t="str">
-        <v/>
-      </c>
-      <c r="F27" t="str">
-        <v>Nao e Campo Calculado</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>Indicadores de Chamados e Workflows</v>
-      </c>
-      <c r="B28" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/IndicadoresdeChamadoseWorkflows/Painel0-Home</v>
-      </c>
-      <c r="C28" t="str">
-        <v>dCalendario; fChamadosEmAberto; fChamadosResolvidos; fWorkflowsEmAberto; fWorkflowsResolvidos</v>
-      </c>
-      <c r="D28" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/workbooks/2227/lineage</v>
-      </c>
-      <c r="E28" t="str">
-        <v>Ano; Ano Fiscal; Data; Dia; Dia da Semana; Dia da Semana ID; Extract (Count); Fiscal Year; Mês; Mês Abr; Mês Fiscal; Mês ID; Mês/Ano; Mês/Ano ID; Período Fiscal ID; Período/FY; Período/FY ID; Semana do Ano; Semana do Ano ID; Semana Fiscal do Ano; Semana Fiscal do Ano ID; Semana Fiscal/Ano ID; Semana/Ano; Semana/Ano ID; Semestre Fiscal / Ano ID; Semestre Fiscal do Ano; Semestre ID; Trimestre Fiscal; Trimestre Fiscal/Ano; Trimestre Fiscal/Ano ID; Assunto; Atribuído ao Usuário; Criador; Data de Conclusão Alvo; Data de Criação; Data Referência; Em nome de; Equipe Atribuída; Fila Atribuída; Fonte; Horas SLA; ID do caso; ID do Caso Relacionado; Prioridade; Solicitado por; Status do caso; Subtópico de RH; Tema de RH; % No Prazo; :Measure Names; Atingiu a Meta; Data de Conclusão Alvo Ajustada; Data de reabertura; Data Referência Resolução; Data/Hora da Primeira Resposta; Data/Hora Resolvida; Dia da Semana Criação; Fila Atribuída (Subequipe); Meta; Número do chamado; Período Fiscal; Qtde Em Atraso; Qtde No Prazo; Reabertos; Status do chamado; Status Prazo Primeiro Atendimento; Tempo de Resolução do Caso (Dias Úteis); Tempo de Trabalho em Dias Úteis; Tempo de trabalho em horas úteis (até agora); Total Atendimentos; Data da Etapa; Data prazo atendimento; Data Referencia; Data/hora início da transação; Dentro do prazo?; Equipe; Etapa de Workflow; Feriado; Formulário de Workflow; Id etapa de workflow; Id Formulário de Workflow; Id Lançamento de Workflow; Nome do Usuário; Referência; Solicitante; Subequipe; % Dentro do Prazo; Atendido Em; Categoria Dia Entrada Wf; Categoria Dia Prazo Atend; Data Prazo Atendimento 2; Data Rescisão; Dentro Prazo?; Efetivado?; Entrada Wf; Entrada Wf 2; Etapa Destino; Etapa Origem; Etapa Wf - Destino; Etapa Wf - Origem; Formulário Wf; Grupo Usuário; Id Formulário Wf; Id Grupo Usuário; Id Log Transação Wf; Id Workflow; Meta WFs; Nome Usuário; Novo Status Dentro Prazo; Prazo Atendimento 1º Dia Útil Próximo Mês; Prazo Atendimento Exceto Abertura Fim De Mês; Qtde Dentro do Prazo; Qtde Fora do Prazo; Status da Meta; Superior Hierárquico; Tempo Atendim Horas Uteis; Tempo Atendimento Hr</v>
-      </c>
-      <c r="F28" t="str">
-        <v>Campo Calculado</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>Indicadores de Chamados e Workflows</v>
-      </c>
-      <c r="B29" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/IndicadoresdeChamadoseWorkflows/Painel0-Home</v>
-      </c>
-      <c r="C29" t="str">
-        <v>dCalendario; fChamadosEmAberto; fChamadosResolvidos; fWorkflowsEmAberto; fWorkflowsResolvidos</v>
-      </c>
-      <c r="D29" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/workbooks/2227/lineage</v>
-      </c>
-      <c r="E29" t="str">
-        <v/>
-      </c>
-      <c r="F29" t="str">
-        <v>Nao e Campo Calculado</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>Visão consolidada</v>
-      </c>
-      <c r="B30" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/Visoconsolidada/Consolidadodedados</v>
-      </c>
-      <c r="C30" t="str">
-        <v>RH - Colaborador Folha; Elegiveis cota aprendiz (Tableau); PCD (Tableau)</v>
-      </c>
-      <c r="D30" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/700/lineage</v>
-      </c>
-      <c r="E30" t="str">
-        <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR; Elegiveis cota aprendiz (Count); Fração p/ Empregado; Função Para Cota Sim; Matrícula; PCD (Count); Qtd. Pcd</v>
-      </c>
-      <c r="F30" t="str">
-        <v>Campo Calculado</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>Visão consolidada</v>
-      </c>
-      <c r="B31" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/Visoconsolidada/Consolidadodedados</v>
-      </c>
-      <c r="C31" t="str">
-        <v>RH - Colaborador Folha; Elegiveis cota aprendiz (Tableau); PCD (Tableau)</v>
-      </c>
-      <c r="D31" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/700/lineage</v>
-      </c>
-      <c r="E31" t="str">
-        <v/>
-      </c>
-      <c r="F31" t="str">
-        <v>Nao e Campo Calculado</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>Zona Posicionamento Salarial</v>
-      </c>
-      <c r="B32" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/ZonaPosicionamentoSalarial/ZonasdePosicionamentoSalarial</v>
-      </c>
-      <c r="C32" t="str">
-        <v>RH - Base_Enios_Tableau; RH - Colaborador Folha</v>
-      </c>
-      <c r="D32" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/52187/lineage; https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage</v>
-      </c>
-      <c r="E32" t="str">
-        <v>Admissão; Cargo; CL; Colaborador; Cpf; Dados gerados em; Diretoria; Dt Competencia; Dt inic cargo atual; Dt nasc; Gênero; Gestor; Grade; HR Reporting; Matrícula; Munic. cl; Nome do cl; Portfolio; Posição Faixa; Região cl; Segmento; Situação; Tipo cl; Uf cl; Zona posicionamento; % Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR</v>
-      </c>
-      <c r="F32" t="str">
-        <v>Campo Calculado</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>Zona Posicionamento Salarial</v>
-      </c>
-      <c r="B33" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/ZonaPosicionamentoSalarial/ZonasdePosicionamentoSalarial</v>
-      </c>
-      <c r="C33" t="str">
-        <v>RH - Base_Enios_Tableau; RH - Colaborador Folha</v>
-      </c>
-      <c r="D33" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/52187/lineage; https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage</v>
-      </c>
-      <c r="E33" t="str">
-        <v/>
-      </c>
-      <c r="F33" t="str">
-        <v>Nao e Campo Calculado</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>Base de Dados Modelo de Trabalho - Home Office</v>
-      </c>
-      <c r="B34" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/BasedeDadosModelodeTrabalho-HomeOffice/BASEOFICIALPARATABLEAU</v>
-      </c>
-      <c r="C34" t="str">
-        <v>RH - Colaborador Folha; RH - Programação de Férias; RH STEP Afastamento; Base_Catracas; Base_Tableau; reserva_mesas_por_colaborador geral</v>
-      </c>
-      <c r="D34" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48035/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48064/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/2183/lineage</v>
-      </c>
-      <c r="E34" t="str">
-        <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR; Cd Cardapio; Cd Centro Custo; Cd Empresa Sodexo; Cd Filial Ficticia; Cd Grupoeconomico; Cd Matricula Diretor Operac; Cd Matricula Gerente Area; Cd Matricula Gerente Regional; Cd Matriz; Cd Período Descanso; Cd Status; Cd Tipo Atuacao; Cd Tipo Servico; Cd Uf; Classificação HR Reporting; Cor Pele; Cpf; Ctps; Ctps Serie; DATABASE; AFAST_CARGO; AFAST_CD_FILIAL; AFAST_CD_SITUACAO; AFAST_CID_DOENCA; AFAST_CID_DOENCA_OFICIAL; AFAST_DSC_DOENCA; AFAST_DSC_MOTIVO_SITUACAO; AFAST_DT_CARGA; AFAST_DT_COMPETENCIA; AFAST_DT_FIM; AFAST_DT_INICIO; AFAST_MATRICULA; AFAST_MOTIVO; AFAST_QT_DIAS_AFASTAMENTO; AFAST_QT_DIAS_AFASTAMENTO_STEP; AFAST_SITUACAO; Competencia; Data Acesso; Email; Empresa; Eqp Id; Equipamento; ES; Hora Acesso; Matricula; Nome; Planilha1 (Count); Qt Acessos; % Conformidade Hibrido Dentro da Meta; % Conformidade Hibrido Fora da Meta; % Conformidade Home 100%; % Conformidade Home Geral; % Conformidade Home Hibrido; :Measure Names; Analise Qt Check-in; Analise Qt Check-in 2; Base_Tableau (Count); Business Unit; Competência; Cor Conformidade; Dias de afastamento no mês; Dias de férias no mês; Dsc Cargo; Dt Admissao; Elegiveis por UF; Email Gestor; Flag Last 6 Month; Flag Mes Atual; Gestor; Matricula Gestor; Modelo de Trabalho; Nm Diretoria; Nm Filial; Nm Segmento; Nome Colaborador; Qt Check-in; Qt Check-in Filtro; Qt Colab Divergente Home 100%; Qt Colab Divergente Home Hibrido; Qt Colaboradores; Qt Colaboradores Filtro; Qt de Check-in; Qt Home Office 100%; Qt Home Office 100% em conformidade; Qt Home Office 100% Não conformidade; Qt Home Office em conformidade; Andar; Cancelado por; Check-in &lt;4; Check-in realizado; Check-out realizado; Data da solicitação; Data de cancelamento; Data do check-in; Data do check-out; Data final; Data inicial; E-mail; Id; Mesa; Plan1 (Count); Planta; Qt Checkin Home Office 100% Divergente; Qt Colab Home Office 100% Divergente; Qt Colab Home Office Hibrido Divergente; Qt de Checkin; Qt Errada Hibrido; Status; Tirou férias no mês?; Total de Check-in; Total de Check-in DIM; Total de Checkin</v>
-      </c>
-      <c r="F34" t="str">
-        <v>Campo Calculado</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>Base de Dados Modelo de Trabalho - Home Office</v>
-      </c>
-      <c r="B35" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/BasedeDadosModelodeTrabalho-HomeOffice/BASEOFICIALPARATABLEAU</v>
-      </c>
-      <c r="C35" t="str">
-        <v>RH - Colaborador Folha; RH - Programação de Férias; RH STEP Afastamento; Base_Catracas; Base_Tableau; reserva_mesas_por_colaborador geral</v>
-      </c>
-      <c r="D35" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48035/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48064/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/2183/lineage</v>
-      </c>
-      <c r="E35" t="str">
-        <v/>
-      </c>
-      <c r="F35" t="str">
-        <v>Nao e Campo Calculado</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>Indicadores de Promoções Internas</v>
-      </c>
-      <c r="B36" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/IndicadoresdePromoesInternas/PromoesInternas</v>
-      </c>
-      <c r="C36" t="str">
-        <v>RH - Colaborador Folha</v>
-      </c>
-      <c r="D36" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage</v>
-      </c>
-      <c r="E36" t="str">
-        <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR</v>
-      </c>
-      <c r="F36" t="str">
-        <v>Campo Calculado</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>Indicadores de Promoções Internas</v>
-      </c>
-      <c r="B37" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/IndicadoresdePromoesInternas/PromoesInternas</v>
-      </c>
-      <c r="C37" t="str">
-        <v>RH - Colaborador Folha</v>
-      </c>
-      <c r="D37" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage</v>
-      </c>
-      <c r="E37" t="str">
-        <v/>
-      </c>
-      <c r="F37" t="str">
-        <v>Nao e Campo Calculado</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="str">
-        <v>Indicadores de Modelo de Trabalho - Home Office</v>
-      </c>
-      <c r="B38" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/IndicadoresdeModelodeTrabalho-HomeOffice_17522412067850/DashboardHomeOffice-Colaboradores</v>
-      </c>
-      <c r="C38" t="str">
-        <v>RH - Colaborador Folha; RH - Programação de Férias; RH STEP Afastamento; Base_Tableau; reserva_mesas_por_colaborador geral</v>
-      </c>
-      <c r="D38" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48035/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48064/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/2169/lineage</v>
-      </c>
-      <c r="E38" t="str">
-        <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR; Cd Cardapio; Cd Centro Custo; Cd Empresa Sodexo; Cd Filial Ficticia; Cd Grupoeconomico; Cd Matricula Diretor Operac; Cd Matricula Gerente Area; Cd Matricula Gerente Regional; Cd Matriz; Cd Período Descanso; Cd Status; Cd Tipo Atuacao; Cd Tipo Servico; Cd Uf; Classificação HR Reporting; Cor Pele; Cpf; Ctps; Ctps Serie; DATABASE; AFAST_CARGO; AFAST_CD_FILIAL; AFAST_CD_SITUACAO; AFAST_CID_DOENCA; AFAST_CID_DOENCA_OFICIAL; AFAST_DSC_DOENCA; AFAST_DSC_MOTIVO_SITUACAO; AFAST_DT_CARGA; AFAST_DT_COMPETENCIA; AFAST_DT_FIM; AFAST_DT_INICIO; AFAST_MATRICULA; AFAST_MOTIVO; AFAST_QT_DIAS_AFASTAMENTO; AFAST_QT_DIAS_AFASTAMENTO_STEP; AFAST_SITUACAO; % Conformidade Hibrido Dentro da Meta; % Conformidade Hibrido Fora da Meta; % Conformidade Home 100%; % Conformidade Home Geral; % Conformidade Home Hibrido; :Measure Names; Analise Qt Check-in; Analise Qt Check-in 2; Base_Tableau (Count); Business Unit; Competência; Cor Conformidade; Dias de afastamento no mês; Dias de férias no mês; Dsc Cargo; Dt Admissao; Elegiveis por UF; Email Gestor; Flag Last 6 Month; Flag Mes Atual; Gestor; Matricula; Matricula Gestor; Modelo de Trabalho; Nm Diretoria; Nm Filial; Nm Segmento; Nome Colaborador; Qt Check-in; Qt Check-in Filtro; Qt Colab Divergente Home 100%; Qt Colab Divergente Home Hibrido; Qt Colaboradores; Qt Colaboradores Filtro; Qt de Check-in; Qt Home Office 100%; Qt Home Office 100% em conformidade; Qt Home Office 100% Não conformidade; Qt Home Office em conformidade; Andar; Cancelado por; Check-in &lt;4; Check-in realizado; Check-out realizado; Competencia; Data da solicitação; Data de cancelamento; Data do check-in; Data do check-out; Data final; Data inicial; E-mail; Id; Mesa; Nome; Plan1 (Count); Planta; Qt Checkin Home Office 100% Divergente; Qt Colab Home Office 100% Divergente; Qt Colab Home Office Hibrido Divergente; Qt Errada Hibrido; Status; Tirou férias no mês?; Total de Check-in; Total de Check-in DIM; Total de Checkin</v>
-      </c>
-      <c r="F38" t="str">
-        <v>Campo Calculado</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="str">
-        <v>Indicadores de Modelo de Trabalho - Home Office</v>
-      </c>
-      <c r="B39" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/IndicadoresdeModelodeTrabalho-HomeOffice_17522412067850/DashboardHomeOffice-Colaboradores</v>
-      </c>
-      <c r="C39" t="str">
-        <v>RH - Colaborador Folha; RH - Programação de Férias; RH STEP Afastamento; Base_Tableau; reserva_mesas_por_colaborador geral</v>
-      </c>
-      <c r="D39" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48035/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48064/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/2169/lineage</v>
-      </c>
-      <c r="E39" t="str">
-        <v/>
-      </c>
-      <c r="F39" t="str">
-        <v>Nao e Campo Calculado</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="str">
-        <v>Painel de Vagas Operacionais</v>
-      </c>
-      <c r="B40" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/PaineldeVagasOperacionais/AnlisesdeVagasOperacionais</v>
-      </c>
-      <c r="C40" t="str">
-        <v>BIVARREDURA - Filial; RH - Colaborador Folha; RH STEP Abertura de Vagas</v>
-      </c>
-      <c r="D40" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/23931/lineage; https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48063/lineage</v>
-      </c>
-      <c r="E40" t="str">
-        <v>[END] Bairro; [END] CEP; [END] Cidade; [END] LATITUDE; [END] Logadouro; [END] LONGITUDE; [END] UF; Cd Cardapio; Cd Centro Custo; Cd Diretoria; Cd Empresa Sodexo; Cd Filial; Cd Filial Ficticia; Cd Grupo Economico; Cd Matricula Diretor Operac; Cd Matricula Gerente Area; Cd Matricula Gerente Regional; Cd Matriz; Cd Regional; Cd Segmento; Cd Tipo Atuacao; Cd Tipo Contrato; Cd Tipo Servico; Cd Uf; CD_BUSINESS_UNIT; Dados migrados (Count); Dt Abertura; Dt Encerramento; Fili Email; Fl Ficticia; Inscricaoestadual; Nm Bairro; Nm Cardapio; Nm Cidade; Nm Diretor Operacional; Nm Diretoria; Nm Empresa Sodexo; Nm Filial; Nm Gerente Area; Nm Gerente Regional; % Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial Colaborador; Cd Grupo CL; Cd Matriz Cardapio; Cd Matriz Compras; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR; Cd Portfolio; CD_CARGO; CD_CARGO_HR_REPORTING; CD_CARGO_VAGA; CD_COTA_APRENDIZ_CBO; CD_ESTR_HIERAR; CD_ESTR_HIERAR_COLAB; CD_FILIAL_COLABORADOR; CD_FILIAL_VAGA; CD_FLEXIVEL_VAGA; CD_SINDICATO; CD_SITUACAO; CD_VAGA; CLASSIFICACAO_HR_REPORTING; COR_PELE; CPF; CTPS</v>
-      </c>
-      <c r="F40" t="str">
-        <v>Campo Calculado</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="str">
-        <v>Painel de Vagas Operacionais</v>
-      </c>
-      <c r="B41" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/PaineldeVagasOperacionais/AnlisesdeVagasOperacionais</v>
-      </c>
-      <c r="C41" t="str">
-        <v>BIVARREDURA - Filial; RH - Colaborador Folha; RH STEP Abertura de Vagas</v>
-      </c>
-      <c r="D41" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/23931/lineage; https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/datasources/48063/lineage</v>
-      </c>
-      <c r="E41" t="str">
-        <v/>
-      </c>
-      <c r="F41" t="str">
-        <v>Nao e Campo Calculado</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="str">
-        <v>Pin People On e Off</v>
-      </c>
-      <c r="B42" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/PinPeopleOneOff/PinPeople</v>
-      </c>
-      <c r="C42" t="str">
-        <v>RH - Colaborador Folha | Projeto : Fonte de Dados Corporativa; tbElegibilidade_Cargo (db_Elegilidade_Cargos)</v>
-      </c>
-      <c r="D42" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/1009/lineage</v>
-      </c>
-      <c r="E42" t="str">
         <v>% Fidelização; % Horas Extras; % Rotatividade; % Rotatividade Acumulada; Bairro; Bh Credito Mes; Bh Descanso; Bh Horas Pagas; Bh Saldo Anterior; Bh Saldo Atual; Cargo Elegivel Jovem Aprendiz; CBO; Cd Business Unit; Cd Cargo; Cd Cargo HR Reporting; Cd Contrato; Cd Cota Aprendiz CBO; Cd Diretoria; Cd Empresa; Cd Estr Hierar; Cd Estr Hierar Colab; Cd Filial; Cd Filial Colaborador; Cd Grupo CL; Cd Grupo Economico; Cd Matriz Cardapio; Cd Matriz Compras; Cd Regional; Cd Segmento; Cd Sindicato; Cd Site; Cd Situacao; Cd SubGrupo CL; Cd Tipo Atuação; Cd Tipo Contrato; Cd Tipo Serviço; CD_FLEXIVEL; CD_HORARIO; CD_STATUS_VAGA; CD_TP_FILIAL_COLABORADOR; Cargo de Confiança; Categoria; Cota Aprendiz; Elegibilidade; Elegibilidade CBO; Grade; ID Elegibilidade Cota JA; Id Nível Hierárquico; Job Family; Job Family Group; Job Title - Inglês; Job Title - Português; Nível Hierárquico; Nível Superior; tbElegibilidade_Cargo (Count)</v>
-      </c>
-      <c r="F42" t="str">
-        <v>Campo Calculado</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="str">
-        <v>Pin People On e Off</v>
-      </c>
-      <c r="B43" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/views/PinPeopleOneOff/PinPeople</v>
-      </c>
-      <c r="C43" t="str">
-        <v>RH - Colaborador Folha | Projeto : Fonte de Dados Corporativa; tbElegibilidade_Cargo (db_Elegilidade_Cargos)</v>
-      </c>
-      <c r="D43" t="str">
-        <v>https://analyticsbi.sodexo.com.br/#/datasources/56353/lineage; https://analyticsbi.sodexo.com.br/#/workbooks/1009/lineage</v>
-      </c>
-      <c r="E43" t="str">
-        <v/>
-      </c>
-      <c r="F43" t="str">
-        <v>Nao e Campo Calculado</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>